<commit_message>
release(v2.0): 2.0.0a7, Phase 5 new skills wave 1 (#1)
Version 2.0.0a6 -> 2.0.0a7 (tools/release.py); goldens regenerated (footer
version only; HTML hashes verified version-only); Hazira samples re-rendered
at SOURCE_DATE_EPOCH=1793059200 (2026-10-27), dashboard adoption tables now
list the Phase 5 packs. Gate OK: 4679 passed on 3.9 and 3.14, coverage 97%,
185 evals, smoke 34 goldens, check-samples 0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011J2b33mikuz2J1RKTx4krR
</commit_message>
<xml_diff>
--- a/samples/2020-09-24-hazira-gas-release-fire/outputs/compliance-crosswalk.xlsx
+++ b/samples/2020-09-24-hazira-gas-release-fire/outputs/compliance-crosswalk.xlsx
@@ -1065,7 +1065,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CGenerated with ProbeMatrix Learnings Coach v2.0.0a6 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</oddFooter>
+    <oddFooter>&amp;CGenerated with ProbeMatrix Learnings Coach v2.0.0a7 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1645,7 +1645,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CGenerated with ProbeMatrix Learnings Coach v2.0.0a6 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</oddFooter>
+    <oddFooter>&amp;CGenerated with ProbeMatrix Learnings Coach v2.0.0a7 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
release(v2.0): 2.0.0a8, Phase 6 new skills wave 2 and library foundation (#1)
Version 2.0.0a7 -> 2.0.0a8 (tools/release.py); goldens regenerated
(PMLC_UPDATE_GOLDEN=1; md diffs version-only, html-golden hashes follow the
footer); Hazira samples re-rendered with the Phase 6 rerender-samples.sh at
SOURCE_DATE_EPOCH=1793145600 (2026-10-28), incl. the Phase 6 packs and
showcases; dashboard, register xlsx and register md regenerated. Sample
diffs are version and date only. Smoke OK (39 fixture packs, 41 Hazira
golden packs), check-samples 0 problems, focused golden/sample tests
175 passed. Full gate run by the orchestrator next.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011J2b33mikuz2J1RKTx4krR
</commit_message>
<xml_diff>
--- a/samples/2020-09-24-hazira-gas-release-fire/outputs/compliance-crosswalk.xlsx
+++ b/samples/2020-09-24-hazira-gas-release-fire/outputs/compliance-crosswalk.xlsx
@@ -1065,7 +1065,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CGenerated with ProbeMatrix Learnings Coach v2.0.0a7 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</oddFooter>
+    <oddFooter>&amp;CGenerated with ProbeMatrix Learnings Coach v2.0.0a8 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1645,7 +1645,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader>&amp;CLearning purposes: not a statutory document · DRAFT</oddHeader>
-    <oddFooter>&amp;CGenerated with ProbeMatrix Learnings Coach v2.0.0a7 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</oddFooter>
+    <oddFooter>&amp;CGenerated with ProbeMatrix Learnings Coach v2.0.0a8 (open source, MIT) from a ProbeMatrix four-level human-factors investigation. ProbeMatrix by Eyekyam: ashley@eyekyam.com</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>